<commit_message>
Ajustar liderazgo territorial y administracion
</commit_message>
<xml_diff>
--- a/public/templates/carga-masiva-dr-jahir.xlsx
+++ b/public/templates/carga-masiva-dr-jahir.xlsx
@@ -154,6 +154,12 @@
     <t>cedula</t>
   </si>
   <si>
+    <t>tipo_registro</t>
+  </si>
+  <si>
+    <t>sector_lider</t>
+  </si>
+  <si>
     <t>telefono</t>
   </si>
   <si>
@@ -196,6 +202,51 @@
     <t>notas</t>
   </si>
   <si>
+    <t>Mariana</t>
+  </si>
+  <si>
+    <t>Suarez</t>
+  </si>
+  <si>
+    <t>1053978521</t>
+  </si>
+  <si>
+    <t>Lider</t>
+  </si>
+  <si>
+    <t>Bajo Tablazo</t>
+  </si>
+  <si>
+    <t>3105550001</t>
+  </si>
+  <si>
+    <t>mariana.suarez@drjahir.com</t>
+  </si>
+  <si>
+    <t>Lider comunitaria</t>
+  </si>
+  <si>
+    <t>Comunidad Bajo Tablazo</t>
+  </si>
+  <si>
+    <t>Lider del sector</t>
+  </si>
+  <si>
+    <t>independiente</t>
+  </si>
+  <si>
+    <t>Puesto Bajo Tablazo</t>
+  </si>
+  <si>
+    <t>bajo tablazo, movilizacion</t>
+  </si>
+  <si>
+    <t>operational</t>
+  </si>
+  <si>
+    <t>Fila de ejemplo para crear una lider.</t>
+  </si>
+  <si>
     <t>Laura</t>
   </si>
   <si>
@@ -205,10 +256,13 @@
     <t>1002458891</t>
   </si>
   <si>
+    <t>Persona</t>
+  </si>
+  <si>
     <t>3105551201</t>
   </si>
   <si>
-    <t>laura.gomez@demo.local</t>
+    <t>laura.gomez@drjahir.com</t>
   </si>
   <si>
     <t>Cra. 24 #19-31</t>
@@ -232,9 +286,6 @@
     <t>salud, mujeres, territorio</t>
   </si>
   <si>
-    <t>operational</t>
-  </si>
-  <si>
     <t>Ejemplo: reemplazar por datos reales.</t>
   </si>
   <si>
@@ -260,9 +311,6 @@
   </si>
   <si>
     <t>Presidente</t>
-  </si>
-  <si>
-    <t>Lider</t>
   </si>
   <si>
     <t>comunidad, rural</t>
@@ -585,25 +633,27 @@
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="28" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
-    <col min="11" max="11" width="24" customWidth="1"/>
-    <col min="12" max="12" width="22" customWidth="1"/>
-    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="9" max="9" width="24" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="13" max="13" width="24" customWidth="1"/>
     <col min="14" max="14" width="22" customWidth="1"/>
-    <col min="15" max="15" width="18" customWidth="1"/>
-    <col min="16" max="16" width="28" customWidth="1"/>
-    <col min="17" max="17" width="10" customWidth="1"/>
-    <col min="18" max="18" width="16" customWidth="1"/>
-    <col min="19" max="19" width="18" customWidth="1"/>
+    <col min="15" max="15" width="22" customWidth="1"/>
+    <col min="16" max="16" width="22" customWidth="1"/>
+    <col min="17" max="17" width="18" customWidth="1"/>
+    <col min="18" max="18" width="28" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
     <col min="20" max="20" width="16" customWidth="1"/>
-    <col min="21" max="21" width="28" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
     <col min="22" max="22" width="16" customWidth="1"/>
-    <col min="23" max="23" width="34" customWidth="1"/>
+    <col min="23" max="23" width="28" customWidth="1"/>
+    <col min="24" max="24" width="16" customWidth="1"/>
+    <col min="25" max="25" width="34" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -629,22 +679,22 @@
         <v>48</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>51</v>
@@ -653,16 +703,16 @@
         <v>52</v>
       </c>
       <c r="P1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>54</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>55</v>
@@ -676,140 +726,233 @@
       <c r="W1" s="1" t="s">
         <v>58</v>
       </c>
+      <c r="X1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G2" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="M2" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="N2" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="O2" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="P2" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q2" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="R2" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="S2" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="T2" s="0"/>
+      <c r="U2" s="0" t="s">
         <v>64</v>
       </c>
-      <c r="H2" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="J2" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="K2" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="L2" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="M2" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="N2" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="O2" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="P2" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q2" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="R2" s="0"/>
-      <c r="S2" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="T2" s="0">
-        <v>84</v>
-      </c>
-      <c r="U2" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="V2" s="0" t="s">
-        <v>71</v>
+      <c r="V2" s="0">
+        <v>96</v>
       </c>
       <c r="W2" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
+      </c>
+      <c r="X2" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="Y2" s="0" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B3" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="E3" s="0"/>
+      <c r="F3" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>81</v>
+      </c>
+      <c r="I3" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="J3" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="M3" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="N3" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="O3" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="P3" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q3" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="R3" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="S3" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="T3" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="U3" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="V3" s="0">
+        <v>84</v>
+      </c>
+      <c r="W3" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="X3" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="C3" s="0" t="s">
-        <v>75</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>76</v>
-      </c>
-      <c r="E3" s="0" t="s">
-        <v>76</v>
-      </c>
-      <c r="F3" s="0"/>
-      <c r="G3" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="H3" s="0" t="s">
+      <c r="Y3" s="0" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" s="0"/>
+      <c r="F4" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="H4" s="0"/>
+      <c r="I4" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="J4" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="K4" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="0" t="s">
+      <c r="L4" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="K3" s="0" t="s">
+      <c r="M4" s="0" t="s">
         <v>37</v>
       </c>
-      <c r="L3" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="M3" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="N3" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="O3" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="P3" s="0" t="s">
+      <c r="N4" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="O4" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="P4" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q4" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="R4" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="Q3" s="0" t="s">
+      <c r="S4" s="0" t="s">
         <v>41</v>
       </c>
-      <c r="R3" s="0"/>
-      <c r="S3" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="T3" s="0">
+      <c r="T4" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="U4" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="V4" s="0">
         <v>90</v>
       </c>
-      <c r="U3" s="0" t="s">
-        <v>82</v>
-      </c>
-      <c r="V3" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="W3" s="0"/>
+      <c r="W4" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="X4" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="Y4" s="0"/>
     </row>
   </sheetData>
 </worksheet>
@@ -831,39 +974,39 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="C2" s="0">
         <v>5</v>
@@ -873,41 +1016,41 @@
       </c>
       <c r="E2" s="0"/>
       <c r="F2" s="0" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C3" s="0"/>
       <c r="D3" s="0"/>
       <c r="E3" s="0" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Conectar mensajeria a proveedores externos
</commit_message>
<xml_diff>
--- a/public/templates/carga-masiva-dr-jahir.xlsx
+++ b/public/templates/carga-masiva-dr-jahir.xlsx
@@ -31,7 +31,7 @@
     <t>Campos obligatorios en Territorio: municipio.</t>
   </si>
   <si>
-    <t>Campos obligatorios en Personas: nombres, apellidos, cedula, municipio.</t>
+    <t>Campos obligatorios en Personas: nombres, apellidos, cedula, municipio. Para cumpleanos usa fecha_nacimiento.</t>
   </si>
   <si>
     <t>Campos obligatorios en Fechas importantes: titulo, mensaje, y fecha exacta o mes/dia.</t>
@@ -169,6 +169,9 @@
     <t>correo</t>
   </si>
   <si>
+    <t>fecha_nacimiento</t>
+  </si>
+  <si>
     <t>direccion</t>
   </si>
   <si>
@@ -223,6 +226,9 @@
     <t>mariana.suarez@drjahir.com</t>
   </si>
   <si>
+    <t>1992-09-21</t>
+  </si>
+  <si>
     <t>Lider comunitaria</t>
   </si>
   <si>
@@ -265,6 +271,9 @@
     <t>laura.gomez@drjahir.com</t>
   </si>
   <si>
+    <t>1990-04-12</t>
+  </si>
+  <si>
     <t>Cra. 24 #19-31</t>
   </si>
   <si>
@@ -299,6 +308,9 @@
   </si>
   <si>
     <t>3105553366</t>
+  </si>
+  <si>
+    <t>1987-12-03</t>
   </si>
   <si>
     <t>Vereda El Cable</t>
@@ -637,23 +649,24 @@
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="28" customWidth="1"/>
-    <col min="9" max="9" width="24" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
-    <col min="13" max="13" width="24" customWidth="1"/>
-    <col min="14" max="14" width="22" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="24" customWidth="1"/>
     <col min="15" max="15" width="22" customWidth="1"/>
     <col min="16" max="16" width="22" customWidth="1"/>
-    <col min="17" max="17" width="18" customWidth="1"/>
-    <col min="18" max="18" width="28" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="16" customWidth="1"/>
-    <col min="21" max="21" width="18" customWidth="1"/>
-    <col min="22" max="22" width="16" customWidth="1"/>
-    <col min="23" max="23" width="28" customWidth="1"/>
-    <col min="24" max="24" width="16" customWidth="1"/>
-    <col min="25" max="25" width="34" customWidth="1"/>
+    <col min="17" max="17" width="22" customWidth="1"/>
+    <col min="18" max="18" width="18" customWidth="1"/>
+    <col min="19" max="19" width="28" customWidth="1"/>
+    <col min="20" max="20" width="10" customWidth="1"/>
+    <col min="21" max="21" width="16" customWidth="1"/>
+    <col min="22" max="22" width="18" customWidth="1"/>
+    <col min="23" max="23" width="16" customWidth="1"/>
+    <col min="24" max="24" width="28" customWidth="1"/>
+    <col min="25" max="25" width="16" customWidth="1"/>
+    <col min="26" max="26" width="34" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -685,19 +698,19 @@
         <v>50</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>52</v>
@@ -709,13 +722,13 @@
         <v>54</v>
       </c>
       <c r="R1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="S1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>56</v>
@@ -732,227 +745,239 @@
       <c r="Y1" s="1" t="s">
         <v>60</v>
       </c>
+      <c r="Z1" s="1" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E2" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="O2" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="P2" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q2" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="R2" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="S2" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="T2" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="U2" s="0"/>
+      <c r="V2" s="0" t="s">
         <v>65</v>
       </c>
-      <c r="F2" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="G2" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="H2" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="I2" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="J2" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K2" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="M2" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="N2" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="O2" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="P2" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q2" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="R2" s="0" t="s">
-        <v>72</v>
-      </c>
-      <c r="S2" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="T2" s="0"/>
-      <c r="U2" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="V2" s="0">
+      <c r="W2" s="0">
         <v>96</v>
       </c>
-      <c r="W2" s="0" t="s">
-        <v>73</v>
-      </c>
       <c r="X2" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Y2" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
+      </c>
+      <c r="Z2" s="0" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E3" s="0"/>
       <c r="F3" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J3" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="K3" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="K3" s="0" t="s">
+      <c r="L3" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="0" t="s">
+      <c r="M3" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="M3" s="0" t="s">
-        <v>65</v>
-      </c>
       <c r="N3" s="0" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="O3" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="P3" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q3" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="R3" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="S3" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="T3" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="U3" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="V3" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="W3" s="0">
         <v>84</v>
       </c>
-      <c r="P3" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q3" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="R3" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="S3" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="T3" s="0" t="s">
-        <v>63</v>
-      </c>
-      <c r="U3" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="V3" s="0">
-        <v>84</v>
-      </c>
-      <c r="W3" s="0" t="s">
-        <v>88</v>
-      </c>
       <c r="X3" s="0" t="s">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="Y3" s="0" t="s">
-        <v>89</v>
+        <v>76</v>
+      </c>
+      <c r="Z3" s="0" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E4" s="0"/>
       <c r="F4" s="0" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H4" s="0"/>
       <c r="I4" s="0" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="J4" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="K4" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="K4" s="0" t="s">
+      <c r="L4" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="L4" s="0" t="s">
+      <c r="M4" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="M4" s="0" t="s">
+      <c r="N4" s="0" t="s">
         <v>37</v>
       </c>
-      <c r="N4" s="0" t="s">
-        <v>95</v>
-      </c>
       <c r="O4" s="0" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="P4" s="0" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="Q4" s="0" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="R4" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="S4" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="S4" s="0" t="s">
+      <c r="T4" s="0" t="s">
         <v>41</v>
       </c>
-      <c r="T4" s="0" t="s">
-        <v>63</v>
-      </c>
       <c r="U4" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="V4" s="0">
+        <v>64</v>
+      </c>
+      <c r="V4" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="W4" s="0" t="s">
-        <v>98</v>
+      <c r="W4" s="0">
+        <v>90</v>
       </c>
       <c r="X4" s="0" t="s">
-        <v>74</v>
-      </c>
-      <c r="Y4" s="0"/>
+        <v>102</v>
+      </c>
+      <c r="Y4" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="Z4" s="0"/>
     </row>
   </sheetData>
 </worksheet>
@@ -974,39 +999,39 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C2" s="0">
         <v>5</v>
@@ -1016,41 +1041,41 @@
       </c>
       <c r="E2" s="0"/>
       <c r="F2" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C3" s="0"/>
       <c r="D3" s="0"/>
       <c r="E3" s="0" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="F3" s="0" t="s">
         <v>48</v>
       </c>
       <c r="G3" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="I3" s="0" t="s">
         <v>117</v>
-      </c>
-      <c r="H3" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="I3" s="0" t="s">
-        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reorganizar administracion y documentos
</commit_message>
<xml_diff>
--- a/public/templates/carga-masiva-dr-jahir.xlsx
+++ b/public/templates/carga-masiva-dr-jahir.xlsx
@@ -9,7 +9,6 @@
     <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
     <sheet name="Territorio" sheetId="2" r:id="rId2"/>
     <sheet name="Personas" sheetId="3" r:id="rId3"/>
-    <sheet name="Fechas importantes" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -22,7 +21,7 @@
     <t>Plantilla de carga masiva - Dr. Jahir</t>
   </si>
   <si>
-    <t>Llena las hojas Territorio, Personas y Fechas importantes. Puedes dejar hojas vacias si no las necesitas.</t>
+    <t>Llena las hojas Territorio y Personas. Puedes dejar hojas vacias si no las necesitas.</t>
   </si>
   <si>
     <t>No cambies los nombres de las hojas ni los encabezados.</t>
@@ -34,13 +33,10 @@
     <t>Campos obligatorios en Personas: nombres, apellidos, cedula, municipio. Para cumpleanos usa fecha_nacimiento.</t>
   </si>
   <si>
-    <t>Campos obligatorios en Fechas importantes: titulo, mensaje, y fecha exacta o mes/dia.</t>
-  </si>
-  <si>
-    <t>Para audiencia_json usa JSON valido, por ejemplo: {"profession":["docente"]}.</t>
-  </si>
-  <si>
-    <t>Al subir el archivo desde Administracion, el sistema actualiza registros existentes por cedula, municipio o titulo.</t>
+    <t>Las fechas importantes se crean desde el modulo Administracion, no desde esta plantilla.</t>
+  </si>
+  <si>
+    <t>Al subir el archivo desde Administracion, el sistema actualiza registros existentes por cedula o municipio.</t>
   </si>
   <si>
     <t>departamento</t>
@@ -326,66 +322,6 @@
   </si>
   <si>
     <t>comunidad, rural</t>
-  </si>
-  <si>
-    <t>titulo</t>
-  </si>
-  <si>
-    <t>tipo_fecha</t>
-  </si>
-  <si>
-    <t>mes</t>
-  </si>
-  <si>
-    <t>dia</t>
-  </si>
-  <si>
-    <t>fecha_exacta</t>
-  </si>
-  <si>
-    <t>canal</t>
-  </si>
-  <si>
-    <t>audiencia_json</t>
-  </si>
-  <si>
-    <t>mensaje</t>
-  </si>
-  <si>
-    <t>activo</t>
-  </si>
-  <si>
-    <t>Dia del maestro</t>
-  </si>
-  <si>
-    <t>profession_day</t>
-  </si>
-  <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>{"profession":["docente","profesor","maestro"]}</t>
-  </si>
-  <si>
-    <t>Gracias por educar y construir territorio. Feliz dia del maestro, {nombre}.</t>
-  </si>
-  <si>
-    <t>si</t>
-  </si>
-  <si>
-    <t>Jornada especial Manizales</t>
-  </si>
-  <si>
-    <t>campaign_day</t>
-  </si>
-  <si>
-    <t>2026-08-10</t>
-  </si>
-  <si>
-    <t>{"municipality":["Manizales"]}</t>
-  </si>
-  <si>
-    <t>Hola {nombre}, te esperamos en la jornada especial de Manizales.</t>
   </si>
 </sst>
 </file>
@@ -478,11 +414,6 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="0" t="s">
-        <v>7</v>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -508,84 +439,84 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="C2" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="D2" s="0" t="s">
         <v>24</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>25</v>
       </c>
       <c r="E2" s="0">
         <v>81</v>
       </c>
       <c r="F2" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="H2" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="I2" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="J2" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="K2" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="L2" s="0" t="s">
         <v>31</v>
-      </c>
-      <c r="L2" s="0" t="s">
-        <v>32</v>
       </c>
       <c r="M2" s="0">
         <v>5.0702</v>
@@ -596,40 +527,40 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="0" t="s">
-        <v>23</v>
-      </c>
       <c r="C3" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="0" t="s">
         <v>33</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>34</v>
       </c>
       <c r="E3" s="0">
         <v>66</v>
       </c>
       <c r="F3" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="H3" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="I3" s="0" t="s">
         <v>37</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="J3" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="J3" s="0" t="s">
+      <c r="K3" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="K3" s="0" t="s">
+      <c r="L3" s="0" t="s">
         <v>40</v>
-      </c>
-      <c r="L3" s="0" t="s">
-        <v>41</v>
       </c>
       <c r="M3" s="0"/>
       <c r="N3" s="0"/>
@@ -671,412 +602,313 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="C2" s="0" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="D2" s="0" t="s">
         <v>64</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="E2" s="0" t="s">
         <v>65</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="F2" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="G2" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="H2" s="0" t="s">
         <v>67</v>
       </c>
-      <c r="G2" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="H2" s="0" t="s">
+      <c r="I2" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="J2" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="L2" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="O2" s="0" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="K2" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="L2" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="M2" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="N2" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="O2" s="0" t="s">
+      <c r="P2" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="P2" s="0" t="s">
+      <c r="Q2" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="Q2" s="0" t="s">
+      <c r="R2" s="0" t="s">
         <v>72</v>
       </c>
-      <c r="R2" s="0" t="s">
+      <c r="S2" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="S2" s="0" t="s">
-        <v>74</v>
-      </c>
       <c r="T2" s="0" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="U2" s="0"/>
       <c r="V2" s="0" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="W2" s="0">
         <v>96</v>
       </c>
       <c r="X2" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="Y2" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="Y2" s="0" t="s">
+      <c r="Z2" s="0" t="s">
         <v>76</v>
-      </c>
-      <c r="Z2" s="0" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="C3" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="D3" s="0" t="s">
         <v>80</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>81</v>
       </c>
       <c r="E3" s="0"/>
       <c r="F3" s="0" t="s">
+        <v>81</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>81</v>
+      </c>
+      <c r="H3" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="G3" s="0" t="s">
-        <v>82</v>
-      </c>
-      <c r="H3" s="0" t="s">
+      <c r="I3" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="J3" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="J3" s="0" t="s">
+      <c r="K3" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="M3" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="N3" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="O3" s="0" t="s">
         <v>85</v>
       </c>
-      <c r="K3" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="L3" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="M3" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="N3" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="O3" s="0" t="s">
+      <c r="P3" s="0" t="s">
         <v>86</v>
       </c>
-      <c r="P3" s="0" t="s">
+      <c r="Q3" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="Q3" s="0" t="s">
+      <c r="R3" s="0" t="s">
         <v>88</v>
       </c>
-      <c r="R3" s="0" t="s">
+      <c r="S3" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="T3" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="U3" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="V3" s="0" t="s">
         <v>89</v>
-      </c>
-      <c r="S3" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="T3" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="U3" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="V3" s="0" t="s">
-        <v>90</v>
       </c>
       <c r="W3" s="0">
         <v>84</v>
       </c>
       <c r="X3" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="Y3" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="Z3" s="0" t="s">
         <v>91</v>
-      </c>
-      <c r="Y3" s="0" t="s">
-        <v>76</v>
-      </c>
-      <c r="Z3" s="0" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="C4" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>95</v>
-      </c>
       <c r="D4" s="0" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E4" s="0"/>
       <c r="F4" s="0" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H4" s="0"/>
       <c r="I4" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="J4" s="0" t="s">
         <v>97</v>
       </c>
-      <c r="J4" s="0" t="s">
+      <c r="K4" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="L4" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="M4" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="N4" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="O4" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="K4" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="L4" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="M4" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="N4" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="O4" s="0" t="s">
+      <c r="P4" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="P4" s="0" t="s">
+      <c r="Q4" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="Q4" s="0" t="s">
-        <v>101</v>
-      </c>
       <c r="R4" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="S4" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="T4" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="U4" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="V4" s="0" t="s">
         <v>89</v>
-      </c>
-      <c r="S4" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="T4" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="U4" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="V4" s="0" t="s">
-        <v>90</v>
       </c>
       <c r="W4" s="0">
         <v>90</v>
       </c>
       <c r="X4" s="0" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Y4" s="0" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Z4" s="0"/>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="38" customWidth="1"/>
-    <col min="8" max="8" width="56" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>113</v>
-      </c>
-      <c r="C2" s="0">
-        <v>5</v>
-      </c>
-      <c r="D2" s="0">
-        <v>15</v>
-      </c>
-      <c r="E2" s="0"/>
-      <c r="F2" s="0" t="s">
-        <v>114</v>
-      </c>
-      <c r="G2" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="H2" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="I2" s="0" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="C3" s="0"/>
-      <c r="D3" s="0"/>
-      <c r="E3" s="0" t="s">
-        <v>120</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="G3" s="0" t="s">
-        <v>121</v>
-      </c>
-      <c r="H3" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="I3" s="0" t="s">
-        <v>117</v>
-      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
Agregar capa operativa en español para cargas
</commit_message>
<xml_diff>
--- a/public/templates/carga-masiva-dr-jahir.xlsx
+++ b/public/templates/carga-masiva-dr-jahir.xlsx
@@ -21,7 +21,7 @@
     <t>Plantilla de carga masiva - Dr. Jahir</t>
   </si>
   <si>
-    <t>Llena las hojas Territorio y Personas. Puedes dejar hojas vacias si no las necesitas.</t>
+    <t>Llena las hojas Territorio y Personas. Tambien puedes subir directamente el archivo votantes.json desde Administracion.</t>
   </si>
   <si>
     <t>No cambies los nombres de las hojas ni los encabezados.</t>
@@ -30,13 +30,16 @@
     <t>Campos obligatorios en Territorio: municipio.</t>
   </si>
   <si>
-    <t>Campos obligatorios en Personas: nombres, apellidos, cedula, municipio. Para cumpleanos usa fecha_nacimiento.</t>
+    <t>Campos obligatorios en Personas: nombres y cedula. Si falta municipio se cargara como Por asignar.</t>
   </si>
   <si>
     <t>Las fechas importantes se crean desde el modulo Administracion, no desde esta plantilla.</t>
   </si>
   <si>
     <t>Al subir el archivo desde Administracion, el sistema actualiza registros existentes por cedula o municipio.</t>
+  </si>
+  <si>
+    <t>Para revisar datos incompletos en Supabase usa la vista operacion_personas_pendientes.</t>
   </si>
   <si>
     <t>departamento</t>
@@ -414,6 +417,11 @@
         <v>6</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -439,84 +447,84 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E2" s="0">
         <v>81</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K2" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L2" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M2" s="0">
         <v>5.0702</v>
@@ -527,40 +535,40 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E3" s="0">
         <v>66</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K3" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L3" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M3" s="0"/>
       <c r="N3" s="0"/>
@@ -602,311 +610,311 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F2" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="K2" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="H2" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="I2" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="J2" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="K2" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="M2" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="N2" s="0" t="s">
-        <v>65</v>
-      </c>
       <c r="O2" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="P2" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q2" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="R2" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="S2" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T2" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="U2" s="0"/>
       <c r="V2" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="W2" s="0">
         <v>96</v>
       </c>
       <c r="X2" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Y2" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Z2" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E3" s="0"/>
       <c r="F3" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K3" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L3" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M3" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N3" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O3" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="P3" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q3" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="R3" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="S3" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="T3" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="U3" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="V3" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="W3" s="0">
         <v>84</v>
       </c>
       <c r="X3" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Y3" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Z3" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E4" s="0"/>
       <c r="F4" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H4" s="0"/>
       <c r="I4" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L4" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M4" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N4" s="0" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="O4" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="P4" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="Q4" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="R4" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="S4" s="0" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="T4" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="U4" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="V4" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="W4" s="0">
         <v>90</v>
       </c>
       <c r="X4" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Y4" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Z4" s="0"/>
     </row>

</xml_diff>